<commit_message>
Recast 2025 State Farm as bundled home+auto on 524.
Only the home share of the Prime State Farm bills hits Unit 1/Unit 2
INSURANCE (50/50, yellow proxy from the Feb unbundled $157.53 / $145.25
charges). Auto share and the Geico *AUTO credit stay personal. No 2025
Travelers found; Sep–Dec State Farm on Prime still open.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/tax_turbo_parts/524 Ferdinand Ave Unit 1.xlsx
+++ b/.cursor/scratch/tax_turbo_parts/524 Ferdinand Ave Unit 1.xlsx
@@ -65,10 +65,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -906,25 +907,25 @@
         <v>0</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>157.53</v>
+        <v>78.76000000000001</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>151.37</v>
+        <v>78.75</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>151.37</v>
+        <v>78.75</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>151.37</v>
+        <v>78.75</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>151.37</v>
+        <v>78.75</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>151.37</v>
+        <v>78.75</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>154.13</v>
+        <v>80.19</v>
       </c>
       <c r="K11" s="3" t="n">
         <v>0</v>
@@ -999,13 +1000,13 @@
       <c r="C13" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="5" t="n">
         <v>66.56</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="5" t="n">
         <v>688.6</v>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="F13" s="5" t="n">
         <v>39.57</v>
       </c>
       <c r="G13" s="2" t="n">
@@ -1014,19 +1015,19 @@
       <c r="H13" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I13" s="4" t="n">
+      <c r="I13" s="5" t="n">
         <v>50.99</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="4" t="n">
+      <c r="K13" s="5" t="n">
         <v>34.86</v>
       </c>
-      <c r="L13" s="4" t="n">
+      <c r="L13" s="5" t="n">
         <v>68.48</v>
       </c>
-      <c r="M13" s="4" t="n">
+      <c r="M13" s="5" t="n">
         <v>32.33</v>
       </c>
       <c r="N13" s="2" t="n">
@@ -1043,40 +1044,40 @@
           <t>VILLAGE WATER AND REFUSE</t>
         </is>
       </c>
-      <c r="C14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="4" t="n">
+      <c r="C14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="5" t="n">
         <v>100.55</v>
       </c>
-      <c r="E14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="4" t="n">
+      <c r="E14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="5" t="n">
         <v>90.67</v>
       </c>
-      <c r="G14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="4" t="n">
+      <c r="G14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="5" t="n">
         <v>112.83</v>
       </c>
-      <c r="I14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="4" t="n">
+      <c r="I14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="5" t="n">
         <v>137.63</v>
       </c>
-      <c r="K14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="4" t="n">
+      <c r="K14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="5" t="n">
         <v>132.76</v>
       </c>
-      <c r="M14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="3" t="n">
+      <c r="M14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O14">
@@ -1090,40 +1091,40 @@
           <t>GAS</t>
         </is>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="C15" s="5" t="n">
         <v>98.56999999999999</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="D15" s="5" t="n">
         <v>133.33</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" s="5" t="n">
         <v>115.82</v>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="F15" s="5" t="n">
         <v>77.8</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="G15" s="5" t="n">
         <v>79.95</v>
       </c>
-      <c r="H15" s="4" t="n">
+      <c r="H15" s="5" t="n">
         <v>48.08</v>
       </c>
-      <c r="I15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="4" t="n">
+      <c r="I15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="5" t="n">
         <v>79.33</v>
       </c>
-      <c r="K15" s="4" t="n">
+      <c r="K15" s="5" t="n">
         <v>36.25</v>
       </c>
-      <c r="L15" s="4" t="n">
+      <c r="L15" s="5" t="n">
         <v>38.22</v>
       </c>
-      <c r="M15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="4" t="n">
+      <c r="M15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="5" t="n">
         <v>139.35</v>
       </c>
       <c r="O15">
@@ -1137,40 +1138,40 @@
           <t>ELECTRIC</t>
         </is>
       </c>
-      <c r="C16" s="3" t="n">
+      <c r="C16" s="4" t="n">
         <v>132.94</v>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D16" s="4" t="n">
         <v>216.44</v>
       </c>
-      <c r="E16" s="3" t="n">
+      <c r="E16" s="4" t="n">
         <v>184.09</v>
       </c>
-      <c r="F16" s="3" t="n">
+      <c r="F16" s="4" t="n">
         <v>60.95</v>
       </c>
-      <c r="G16" s="3" t="n">
+      <c r="G16" s="4" t="n">
         <v>83.76000000000001</v>
       </c>
-      <c r="H16" s="3" t="n">
+      <c r="H16" s="4" t="n">
         <v>69.69</v>
       </c>
-      <c r="I16" s="3" t="n">
+      <c r="I16" s="4" t="n">
         <v>164.88</v>
       </c>
-      <c r="J16" s="3" t="n">
+      <c r="J16" s="4" t="n">
         <v>203.43</v>
       </c>
-      <c r="K16" s="3" t="n">
+      <c r="K16" s="4" t="n">
         <v>187.63</v>
       </c>
-      <c r="L16" s="3" t="n">
+      <c r="L16" s="4" t="n">
         <v>139.78</v>
       </c>
-      <c r="M16" s="3" t="n">
+      <c r="M16" s="4" t="n">
         <v>71.29000000000001</v>
       </c>
-      <c r="N16" s="3" t="n">
+      <c r="N16" s="4" t="n">
         <v>50.38</v>
       </c>
       <c r="O16">
@@ -1722,9 +1723,9 @@
     </row>
     <row r="29"/>
     <row r="30">
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>§121 residence through sale 2025-12-18. Nicor large / water 50/50 CONFIRMED. March HD + remaining HD/Lowe’s/IKEA 524-share → EXTERIOR REPAIRS (U1 $981.39). ELECTRIC yellow — REMIND JACOB: double-check ComEd with Megan (checking ACH INDN Megan Gerrard $1,565.26; paid ACH and/or check?). Internet still $0 on this tab (Prime ATT on Unit 2). Not tax advice.</t>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>§121 residence through sale 2025-12-18. Nicor large / water 50/50 CONFIRMED. March HD + remaining HD/Lowe’s/IKEA 524-share → EXTERIOR REPAIRS (U1 $981.39). ELECTRIC yellow — REMIND JACOB: double-check ComEd with Megan (checking ACH INDN Megan Gerrard $1,565.26; paid ACH and/or check?). Internet still $0 on this tab (Prime ATT on Unit 2). State Farm: bundled home+auto (was Travelers home / Geico auto). Only HOME share on this INSURANCE line (50/50 with Unit 2, yellow proxy). Auto + Geico credit personal. Not tax advice.</t>
         </is>
       </c>
     </row>

</xml_diff>